<commit_message>
docs(template): human-readable Excel headers + key row + blanks + autofilter
- Row educator titles; row 2 field keys for future import; banner + examples + spare empty rows
- Column_reference matches titles; How_to_use explains layout

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/seaweed-observations-import-template.xlsx
+++ b/public/templates/seaweed-observations-import-template.xlsx
@@ -8,6 +8,9 @@
     <sheet name="Allowed_codes" sheetId="3" r:id="rId3"/>
     <sheet name="Column_reference" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Observations'!A1:Z20</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -400,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A34"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -417,7 +420,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>WHO: Fill one sheet ("Observations") and email the file back (or upload when the team enables file import).</v>
+        <v>OBSERVATIONS SHEET LAYOUT</v>
       </c>
     </row>
     <row r="4">
@@ -427,379 +430,374 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ONE ROW = ONE observation in the database.</v>
+        <v>Row 1 — Column titles: use these to know what goes in each column.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v xml:space="preserve">  • If you weigh a "green" sample and a "red" sample the same day, use TWO rows (same date/time/location, different species and wet_mass_grams).</v>
+        <v>Row 2 — Technical field names: keep this row for automated import later; you can hide row 2 in Excel (Format → Hide) if it distracts you.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v xml:space="preserve">  • If you record only combined total limu mass for a whole system, use one row with species = other (see examples).</v>
+        <v>Row 3 — Reminder banner; then sample rows you should delete.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>Empty rows below are for your data — add more rows in Excel as needed.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>REQUIRED COLUMNS</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">  date — Use YYYY-MM-DD (e.g. 2026-05-12).</v>
+        <v>WHO: Fill "Observations" and email the file back (or upload when the team enables file import).</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v xml:space="preserve">  time — 24-hour HH:MM (e.g. 09:00). If unknown, use 09:00.</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">  observer — Your name as you want it stored.</v>
+        <v>ONE ROW = ONE observation in the database.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v xml:space="preserve">  location — Copy the short code from sheet "Allowed_codes" (e.g. fhw205_large_growth_chamber).</v>
+        <v xml:space="preserve">  • Green + red sample same day → TWO rows (same date, time, location; different species codes and wet masses).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  species — Copy code from "Allowed_codes". Green chamber sample → often ogo_manuea; red sample → often lepe_lepe; system total → other.</v>
+        <v xml:space="preserve">  • Whole-system total mass only → one row, species code "other" (see Allowed_codes + examples).</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v/>
+        <v xml:space="preserve">  • Always copy location &amp; species codes from "Allowed_codes".</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CORE MEASUREMENTS (use what you have; leave cells blank if not measured)</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">  wet_mass_grams — Wet biomass in grams.</v>
+        <v>REQUIRED FOR EACH ROW</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">  salinity_ppt — Salinity in ppt at the same session as the weigh-in, if you measured it.</v>
+        <v xml:space="preserve">  Date (row 1 title "Date…") — YYYY-MM-DD. Time — 24-hour HH:MM. Observer — your name.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v xml:space="preserve">  Location code — e.g. fhw205_large_growth_chamber. Species code — e.g. ogo_manuea or lepe_lepe.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>OPTIONAL — water quality / system</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v xml:space="preserve">  temperature + temperature_unit (F or C), ph, dissolved_oxygen_mg_l</v>
+        <v>CORE MEASUREMENTS (leave blank if not measured)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  container_volume + container_volume_unit (gallons or liters)</v>
+        <v xml:space="preserve">  Wet mass (g), Salinity (ppt), and any optional water-quality / lighting columns.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  Lighting: light_schedule_start/end (HH:MM), light_white_percent, light_red_percent, light_blue_percent (0–100).</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  Interventions: water_exchange_percent, water_exchange_source, nutrients_added</v>
+        <v>OPTIONAL — water quality / system</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v xml:space="preserve">  Temperature + unit (F or C), pH, dissolved O₂, container volume + unit, lighting %, water exchange, nutrients.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>NOTES</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  color_description, health_notes, general_notes — free text.</v>
+        <v>NOTES</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  sensor_issues — TRUE or FALSE (equipment acting oddly).</v>
+        <v xml:space="preserve">  Color, health, and session notes — free text. Sensor issues — TRUE or FALSE. Reliability — see Allowed_codes.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  data_reliability — reliable | uncertain | flagged (see Allowed_codes).</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
+        <v>TIP: Green + red sample same day = two rows (same date/time/location; different species and mass).</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>TIP: Ken often sends Initial / Day 2 / Day 6 tables — each date gets new rows; same session can share time and salinity on both species rows.</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v/>
+        <v>After entering data, delete the example rows. Keep row 1 + row 2 headers.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>After entering data, DELETE the three example rows in "Observations" before sending the file.</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
         <v>Version: generated from repo scripts. Lists match src/types/observation.ts.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z20"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="21.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="21.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" customWidth="1"/>
-    <col min="17" max="17" width="17.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="21.83203125" customWidth="1"/>
-    <col min="21" max="21" width="15.83203125" customWidth="1"/>
-    <col min="22" max="22" width="17.83203125" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="13.83203125" customWidth="1"/>
-    <col min="25" max="25" width="13.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="27.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="27.83203125" customWidth="1"/>
+    <col min="13" max="13" width="33.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="20.83203125" customWidth="1"/>
+    <col min="16" max="16" width="25.83203125" customWidth="1"/>
+    <col min="17" max="17" width="23.83203125" customWidth="1"/>
+    <col min="18" max="18" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="26.83203125" customWidth="1"/>
+    <col min="20" max="20" width="30.83203125" customWidth="1"/>
+    <col min="21" max="21" width="24.83203125" customWidth="1"/>
+    <col min="22" max="22" width="27.83203125" customWidth="1"/>
+    <col min="23" max="23" width="21.83203125" customWidth="1"/>
+    <col min="24" max="24" width="30.83203125" customWidth="1"/>
+    <col min="25" max="25" width="32.83203125" customWidth="1"/>
+    <col min="26" max="26" width="44.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>date</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="B1" t="str">
-        <v>time</v>
+        <v>Time (24-hour HH:MM)</v>
       </c>
       <c r="C1" t="str">
-        <v>observer</v>
+        <v>Observer (your name)</v>
       </c>
       <c r="D1" t="str">
-        <v>location</v>
+        <v>Location code</v>
       </c>
       <c r="E1" t="str">
-        <v>species</v>
+        <v>Species code</v>
       </c>
       <c r="F1" t="str">
-        <v>wet_mass_grams</v>
+        <v>Wet mass (grams)</v>
       </c>
       <c r="G1" t="str">
-        <v>salinity_ppt</v>
+        <v>Salinity (ppt)</v>
       </c>
       <c r="H1" t="str">
-        <v>temperature</v>
+        <v>Temperature (number)</v>
       </c>
       <c r="I1" t="str">
-        <v>temperature_unit</v>
+        <v>Temperature unit (F or C)</v>
       </c>
       <c r="J1" t="str">
-        <v>ph</v>
+        <v>pH</v>
       </c>
       <c r="K1" t="str">
-        <v>dissolved_oxygen_mg_l</v>
+        <v>Dissolved oxygen (mg/L)</v>
       </c>
       <c r="L1" t="str">
-        <v>container_volume</v>
+        <v>Container volume (number)</v>
       </c>
       <c r="M1" t="str">
-        <v>container_volume_unit</v>
+        <v>Volume unit (gallons or liters)</v>
       </c>
       <c r="N1" t="str">
-        <v>light_schedule_start</v>
+        <v>Lights on (HH:MM)</v>
       </c>
       <c r="O1" t="str">
-        <v>light_schedule_end</v>
+        <v>Lights off (HH:MM)</v>
       </c>
       <c r="P1" t="str">
-        <v>light_white_percent</v>
+        <v>Light — white % (0–100)</v>
       </c>
       <c r="Q1" t="str">
-        <v>light_red_percent</v>
+        <v>Light — red % (0–100)</v>
       </c>
       <c r="R1" t="str">
-        <v>light_blue_percent</v>
+        <v>Light — blue % (0–100)</v>
       </c>
       <c r="S1" t="str">
-        <v>water_exchange_percent</v>
+        <v>Water exchange % (0–100)</v>
       </c>
       <c r="T1" t="str">
-        <v>water_exchange_source</v>
+        <v>Water exchange source (text)</v>
       </c>
       <c r="U1" t="str">
-        <v>nutrients_added</v>
+        <v>Nutrients added (text)</v>
       </c>
       <c r="V1" t="str">
-        <v>color_description</v>
+        <v>Color / appearance (text)</v>
       </c>
       <c r="W1" t="str">
-        <v>health_notes</v>
+        <v>Health notes (text)</v>
       </c>
       <c r="X1" t="str">
-        <v>general_notes</v>
+        <v>Session / setup notes (text)</v>
       </c>
       <c r="Y1" t="str">
-        <v>sensor_issues</v>
+        <v>Sensor issues? (TRUE or FALSE)</v>
       </c>
       <c r="Z1" t="str">
-        <v>data_reliability</v>
+        <v>Reliability (reliable / uncertain / flagged)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-12</v>
+        <v>date</v>
       </c>
       <c r="B2" t="str">
-        <v>09:00</v>
+        <v>time</v>
       </c>
       <c r="C2" t="str">
-        <v>Ken Kozuma</v>
+        <v>observer</v>
       </c>
       <c r="D2" t="str">
-        <v>fhw205_large_growth_chamber</v>
+        <v>location</v>
       </c>
       <c r="E2" t="str">
-        <v>ogo_manuea</v>
-      </c>
-      <c r="F2">
-        <v>15.6</v>
-      </c>
-      <c r="G2">
-        <v>27.5</v>
+        <v>species</v>
+      </c>
+      <c r="F2" t="str">
+        <v>wet_mass_grams</v>
+      </c>
+      <c r="G2" t="str">
+        <v>salinity_ppt</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>temperature</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>temperature_unit</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>ph</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>dissolved_oxygen_mg_l</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>container_volume</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>container_volume_unit</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>light_schedule_start</v>
       </c>
       <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2">
-        <v>3</v>
-      </c>
-      <c r="Q2">
-        <v>3</v>
-      </c>
-      <c r="R2">
-        <v>3</v>
+        <v>light_schedule_end</v>
+      </c>
+      <c r="P2" t="str">
+        <v>light_white_percent</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>light_red_percent</v>
+      </c>
+      <c r="R2" t="str">
+        <v>light_blue_percent</v>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>water_exchange_percent</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>water_exchange_source</v>
       </c>
       <c r="U2" t="str">
-        <v/>
+        <v>nutrients_added</v>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>color_description</v>
       </c>
       <c r="W2" t="str">
-        <v/>
+        <v>health_notes</v>
       </c>
       <c r="X2" t="str">
-        <v>Day 6 — DELETE this row and add your own.</v>
+        <v>general_notes</v>
       </c>
       <c r="Y2" t="str">
-        <v>FALSE</v>
+        <v>sensor_issues</v>
       </c>
       <c r="Z2" t="str">
-        <v>reliable</v>
+        <v>data_reliability</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-12</v>
+        <v>▼ Example rows only — delete before sending your file ▼</v>
       </c>
       <c r="B3" t="str">
-        <v>09:01</v>
+        <v/>
       </c>
       <c r="C3" t="str">
-        <v>Ken Kozuma</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>fhw205_large_growth_chamber</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>lepe_lepe</v>
-      </c>
-      <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
-        <v>27.5</v>
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -853,10 +851,10 @@
         <v/>
       </c>
       <c r="Y3" t="str">
-        <v>FALSE</v>
+        <v/>
       </c>
       <c r="Z3" t="str">
-        <v>reliable</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -864,22 +862,22 @@
         <v>2026-05-12</v>
       </c>
       <c r="B4" t="str">
-        <v>10:00</v>
+        <v>09:00</v>
       </c>
       <c r="C4" t="str">
         <v>Ken Kozuma</v>
       </c>
       <c r="D4" t="str">
-        <v>main_500gal_tank</v>
+        <v>fhw205_large_growth_chamber</v>
       </c>
       <c r="E4" t="str">
-        <v>other</v>
+        <v>ogo_manuea</v>
       </c>
       <c r="F4">
-        <v>244.4</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
+        <v>15.6</v>
+      </c>
+      <c r="G4">
+        <v>27.5</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -905,14 +903,14 @@
       <c r="O4" t="str">
         <v/>
       </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
-        <v/>
+      <c r="P4">
+        <v>3</v>
+      </c>
+      <c r="Q4">
+        <v>3</v>
+      </c>
+      <c r="R4">
+        <v>3</v>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -930,18 +928,1299 @@
         <v/>
       </c>
       <c r="X4" t="str">
-        <v>Example: total mixed biomass for main system (one row). DELETE before send.</v>
+        <v>Day 6 — DELETE this row and add your own.</v>
       </c>
       <c r="Y4" t="str">
         <v>FALSE</v>
       </c>
       <c r="Z4" t="str">
+        <v>reliable</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-05-12</v>
+      </c>
+      <c r="B5" t="str">
+        <v>09:01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Ken Kozuma</v>
+      </c>
+      <c r="D5" t="str">
+        <v>fhw205_large_growth_chamber</v>
+      </c>
+      <c r="E5" t="str">
+        <v>lepe_lepe</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5">
+        <v>27.5</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Z5" t="str">
+        <v>reliable</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-05-12</v>
+      </c>
+      <c r="B6" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ken Kozuma</v>
+      </c>
+      <c r="D6" t="str">
+        <v>main_500gal_tank</v>
+      </c>
+      <c r="E6" t="str">
+        <v>other</v>
+      </c>
+      <c r="F6">
+        <v>244.4</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v>Example: total mixed biomass for main system (one row). DELETE before send.</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Z6" t="str">
         <v>uncertain</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:Z20"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1230,28 +2509,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C27"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="52.83203125" customWidth="1"/>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>column_name</v>
+        <v>Excel column title (row 1)</v>
       </c>
       <c r="B1" t="str">
-        <v>meaning</v>
+        <v>Field key (row 2)</v>
       </c>
       <c r="C1" t="str">
-        <v>example</v>
+        <v>Example</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Date (YYYY-MM-DD)</v>
+      </c>
+      <c r="B2" t="str">
         <v>date</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Collection date</v>
       </c>
       <c r="C2" t="str">
         <v>2026-05-12</v>
@@ -1259,10 +2538,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Time (24-hour HH:MM)</v>
+      </c>
+      <c r="B3" t="str">
         <v>time</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Time of reading (24h)</v>
       </c>
       <c r="C3" t="str">
         <v>09:00</v>
@@ -1270,10 +2549,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Observer (your name)</v>
+      </c>
+      <c r="B4" t="str">
         <v>observer</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Person recording</v>
       </c>
       <c r="C4" t="str">
         <v>Ken Kozuma</v>
@@ -1281,10 +2560,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Location code</v>
+      </c>
+      <c r="B5" t="str">
         <v>location</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Site code from Allowed_codes</v>
       </c>
       <c r="C5" t="str">
         <v>castle_outdoor_tumble_tank</v>
@@ -1292,10 +2571,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Species code</v>
+      </c>
+      <c r="B6" t="str">
         <v>species</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Taxon or "other" for totals</v>
       </c>
       <c r="C6" t="str">
         <v>ogo_manuea</v>
@@ -1303,10 +2582,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Wet mass (grams)</v>
+      </c>
+      <c r="B7" t="str">
         <v>wet_mass_grams</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Wet mass (g)</v>
       </c>
       <c r="C7" t="str">
         <v>15.6</v>
@@ -1314,10 +2593,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Salinity (ppt)</v>
+      </c>
+      <c r="B8" t="str">
         <v>salinity_ppt</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Salinity (ppt)</v>
       </c>
       <c r="C8" t="str">
         <v>27.5</v>
@@ -1325,10 +2604,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Temperature (number)</v>
+      </c>
+      <c r="B9" t="str">
         <v>temperature</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Number only</v>
       </c>
       <c r="C9" t="str">
         <v>71.6</v>
@@ -1336,10 +2615,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Temperature unit (F or C)</v>
+      </c>
+      <c r="B10" t="str">
         <v>temperature_unit</v>
-      </c>
-      <c r="B10" t="str">
-        <v>F or C</v>
       </c>
       <c r="C10" t="str">
         <v>F</v>
@@ -1347,10 +2626,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>pH</v>
+      </c>
+      <c r="B11" t="str">
         <v>ph</v>
-      </c>
-      <c r="B11" t="str">
-        <v>pH reading</v>
       </c>
       <c r="C11" t="str">
         <v>8.2</v>
@@ -1358,10 +2637,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>Dissolved oxygen (mg/L)</v>
+      </c>
+      <c r="B12" t="str">
         <v>dissolved_oxygen_mg_l</v>
-      </c>
-      <c r="B12" t="str">
-        <v>DO mg/L</v>
       </c>
       <c r="C12" t="str">
         <v>8.1</v>
@@ -1369,10 +2648,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>Container volume (number)</v>
+      </c>
+      <c r="B13" t="str">
         <v>container_volume</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Number only</v>
       </c>
       <c r="C13" t="str">
         <v>2</v>
@@ -1380,10 +2659,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Volume unit (gallons or liters)</v>
+      </c>
+      <c r="B14" t="str">
         <v>container_volume_unit</v>
-      </c>
-      <c r="B14" t="str">
-        <v>gallons or liters</v>
       </c>
       <c r="C14" t="str">
         <v>gallons</v>
@@ -1391,10 +2670,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>Lights on (HH:MM)</v>
+      </c>
+      <c r="B15" t="str">
         <v>light_schedule_start</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Lights on HH:MM</v>
       </c>
       <c r="C15" t="str">
         <v>08:00</v>
@@ -1402,10 +2681,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>Lights off (HH:MM)</v>
+      </c>
+      <c r="B16" t="str">
         <v>light_schedule_end</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Lights off HH:MM</v>
       </c>
       <c r="C16" t="str">
         <v>18:00</v>
@@ -1413,10 +2692,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v>Light — white % (0–100)</v>
+      </c>
+      <c r="B17" t="str">
         <v>light_white_percent</v>
-      </c>
-      <c r="B17" t="str">
-        <v>0–100</v>
       </c>
       <c r="C17" t="str">
         <v>3</v>
@@ -1424,10 +2703,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>Light — red % (0–100)</v>
+      </c>
+      <c r="B18" t="str">
         <v>light_red_percent</v>
-      </c>
-      <c r="B18" t="str">
-        <v>0–100</v>
       </c>
       <c r="C18" t="str">
         <v>3</v>
@@ -1435,10 +2714,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>Light — blue % (0–100)</v>
+      </c>
+      <c r="B19" t="str">
         <v>light_blue_percent</v>
-      </c>
-      <c r="B19" t="str">
-        <v>0–100</v>
       </c>
       <c r="C19" t="str">
         <v>3</v>
@@ -1446,10 +2725,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>Water exchange % (0–100)</v>
+      </c>
+      <c r="B20" t="str">
         <v>water_exchange_percent</v>
-      </c>
-      <c r="B20" t="str">
-        <v>0–100</v>
       </c>
       <c r="C20" t="str">
         <v>25</v>
@@ -1457,10 +2736,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>Water exchange source (text)</v>
+      </c>
+      <c r="B21" t="str">
         <v>water_exchange_source</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Text</v>
       </c>
       <c r="C21" t="str">
         <v>main aquaponic system</v>
@@ -1468,10 +2747,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>Nutrients added (text)</v>
+      </c>
+      <c r="B22" t="str">
         <v>nutrients_added</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Text</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -1479,10 +2758,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Color / appearance (text)</v>
+      </c>
+      <c r="B23" t="str">
         <v>color_description</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Text</v>
       </c>
       <c r="C23" t="str">
         <v>Outdoor full color</v>
@@ -1490,10 +2769,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>Health notes (text)</v>
+      </c>
+      <c r="B24" t="str">
         <v>health_notes</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Text</v>
       </c>
       <c r="C24" t="str">
         <v/>
@@ -1501,10 +2780,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>Session / setup notes (text)</v>
+      </c>
+      <c r="B25" t="str">
         <v>general_notes</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Text</v>
       </c>
       <c r="C25" t="str">
         <v>Day 6 follow-up…</v>
@@ -1512,10 +2791,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>Sensor issues? (TRUE or FALSE)</v>
+      </c>
+      <c r="B26" t="str">
         <v>sensor_issues</v>
-      </c>
-      <c r="B26" t="str">
-        <v>TRUE or FALSE</v>
       </c>
       <c r="C26" t="str">
         <v>FALSE</v>
@@ -1523,10 +2802,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>Reliability (reliable / uncertain / flagged)</v>
+      </c>
+      <c r="B27" t="str">
         <v>data_reliability</v>
-      </c>
-      <c r="B27" t="str">
-        <v>reliable / uncertain / flagged</v>
       </c>
       <c r="C27" t="str">
         <v>reliable</v>

</xml_diff>